<commit_message>
Update Newman API test results - Jenkins build 9
</commit_message>
<xml_diff>
--- a/reports/ERPNext-API-Test-Results.xlsx
+++ b/reports/ERPNext-API-Test-Results.xlsx
@@ -580,7 +580,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
@@ -603,7 +603,7 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s">
         <v>9</v>
@@ -626,7 +626,7 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
         <v>9</v>
@@ -649,7 +649,7 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>198</v>
+        <v>156</v>
       </c>
       <c r="G5" t="s">
         <v>9</v>
@@ -672,7 +672,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
         <v>9</v>
@@ -695,7 +695,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
         <v>9</v>
@@ -718,7 +718,7 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G8" t="s">
         <v>9</v>
@@ -741,7 +741,7 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G9" t="s">
         <v>9</v>
@@ -797,7 +797,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -814,7 +814,7 @@
         <v>9</v>
       </c>
       <c r="E3">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -831,7 +831,7 @@
         <v>9</v>
       </c>
       <c r="E4">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -848,7 +848,7 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -865,7 +865,7 @@
         <v>9</v>
       </c>
       <c r="E6">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -882,7 +882,7 @@
         <v>9</v>
       </c>
       <c r="E7">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -899,7 +899,7 @@
         <v>9</v>
       </c>
       <c r="E8">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -916,7 +916,7 @@
         <v>9</v>
       </c>
       <c r="E9">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -933,7 +933,7 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>79</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -950,7 +950,7 @@
         <v>9</v>
       </c>
       <c r="E11">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -967,7 +967,7 @@
         <v>9</v>
       </c>
       <c r="E12">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -984,7 +984,7 @@
         <v>9</v>
       </c>
       <c r="E13">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1001,7 +1001,7 @@
         <v>9</v>
       </c>
       <c r="E14">
-        <v>78</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1018,7 +1018,7 @@
         <v>9</v>
       </c>
       <c r="E15">
-        <v>78</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1035,7 +1035,7 @@
         <v>9</v>
       </c>
       <c r="E16">
-        <v>78</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1052,7 +1052,7 @@
         <v>9</v>
       </c>
       <c r="E17">
-        <v>198</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1069,7 +1069,7 @@
         <v>9</v>
       </c>
       <c r="E18">
-        <v>198</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1086,7 +1086,7 @@
         <v>9</v>
       </c>
       <c r="E19">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>9</v>
       </c>
       <c r="E20">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1120,7 +1120,7 @@
         <v>9</v>
       </c>
       <c r="E21">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1137,7 +1137,7 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>9</v>
       </c>
       <c r="E23">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1171,7 +1171,7 @@
         <v>9</v>
       </c>
       <c r="E24">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1188,7 +1188,7 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1205,7 +1205,7 @@
         <v>9</v>
       </c>
       <c r="E26">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1222,7 +1222,7 @@
         <v>9</v>
       </c>
       <c r="E27">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1239,7 +1239,7 @@
         <v>9</v>
       </c>
       <c r="E28">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1256,7 +1256,7 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1273,7 +1273,7 @@
         <v>9</v>
       </c>
       <c r="E30">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1290,7 +1290,7 @@
         <v>9</v>
       </c>
       <c r="E31">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>